<commit_message>
Feat: Layout Finances revu + photo agent Firebase Storage + KPI libellés originaux
- FinancesPage : Vue mensuelle + Bilan annuel côte à côte (xl:grid-cols-2)
- Sections du bas : CSS columns sans trou (columns-1 xl:columns-2 + break-inside-avoid)
- KPI libellés exacts de la version originale (Frais agence, Ont payé/N'ont pas payé, Impayés bruts/Trop-perçus)
- Contrôle croisé : suppression barres de progression (max-h-52 overflow-y-auto retirés)
- AgentEditorModal : upload photo vers Firebase Storage (URL permanente) au lieu de blob URL temporaire
- storage.rules : ajout règle agents/{agentId}/{fileName}
- vite.config.ts : port 3001 (évite conflit avec ancienne version)
- DataPage : fallback startDate → '2020-01-01' pour éviter creux artificiels sur graphique

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import_data/liste locataires orchestra.xlsx
+++ b/import_data/liste locataires orchestra.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49b600b6b06b0bc0/Bureau/beeboxlaon-original/import_data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_DAF9398D826181017B7C26559EA70443014B3403" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F02DAEBD-842B-46F0-AF44-3464A21A3F35}"/>
+  <bookViews>
+    <workbookView xWindow="33345" yWindow="2685" windowWidth="24645" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Feuille 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Feuille 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -46,9 +55,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0053</t>
     </r>
@@ -69,9 +80,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0057</t>
     </r>
@@ -89,9 +102,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0059</t>
     </r>
@@ -109,9 +124,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0028</t>
     </r>
@@ -126,9 +143,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0012</t>
     </r>
@@ -146,9 +165,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0060</t>
     </r>
@@ -163,9 +184,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0003</t>
     </r>
@@ -183,9 +206,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0036</t>
     </r>
@@ -203,9 +228,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0010</t>
     </r>
@@ -223,9 +250,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0013</t>
     </r>
@@ -243,9 +272,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0029</t>
     </r>
@@ -263,9 +294,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0019</t>
     </r>
@@ -283,9 +316,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0026</t>
     </r>
@@ -300,9 +335,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0005</t>
     </r>
@@ -317,9 +354,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0052</t>
     </r>
@@ -337,9 +376,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0051</t>
     </r>
@@ -354,9 +395,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0058</t>
     </r>
@@ -371,9 +414,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0018</t>
     </r>
@@ -391,9 +436,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0022</t>
     </r>
@@ -408,9 +455,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0031</t>
     </r>
@@ -425,9 +474,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0040</t>
     </r>
@@ -442,9 +493,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0024</t>
     </r>
@@ -459,9 +512,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0023</t>
     </r>
@@ -479,9 +534,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0006</t>
     </r>
@@ -499,9 +556,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0059</t>
     </r>
@@ -516,9 +575,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0051</t>
     </r>
@@ -536,9 +597,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0035</t>
     </r>
@@ -553,9 +616,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0042</t>
     </r>
@@ -573,9 +638,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0001</t>
     </r>
@@ -593,9 +660,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0032</t>
     </r>
@@ -613,9 +682,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0015</t>
     </r>
@@ -630,9 +701,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0043</t>
     </r>
@@ -650,9 +723,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0044</t>
     </r>
@@ -667,9 +742,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0036</t>
     </r>
@@ -684,9 +761,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0008</t>
     </r>
@@ -704,9 +783,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0045</t>
     </r>
@@ -724,9 +805,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0034</t>
     </r>
@@ -744,9 +827,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0017</t>
     </r>
@@ -764,9 +849,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0021</t>
     </r>
@@ -781,9 +868,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0041</t>
     </r>
@@ -801,9 +890,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0029</t>
     </r>
@@ -821,9 +912,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0061</t>
     </r>
@@ -841,9 +934,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0046</t>
     </r>
@@ -858,9 +953,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0047</t>
     </r>
@@ -872,9 +969,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0031</t>
     </r>
@@ -892,9 +991,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0025</t>
     </r>
@@ -912,9 +1013,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0006</t>
     </r>
@@ -929,9 +1032,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0048</t>
     </r>
@@ -946,9 +1051,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0049</t>
     </r>
@@ -963,9 +1070,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0014</t>
     </r>
@@ -980,9 +1089,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0023</t>
     </r>
@@ -990,9 +1101,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0001</t>
     </r>
@@ -1010,9 +1123,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0037</t>
     </r>
@@ -1027,9 +1142,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0036</t>
     </r>
@@ -1044,9 +1161,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0013</t>
     </r>
@@ -1064,9 +1183,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0015</t>
     </r>
@@ -1081,9 +1202,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0028</t>
     </r>
@@ -1101,9 +1224,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0027</t>
     </r>
@@ -1118,9 +1243,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0010</t>
     </r>
@@ -1138,9 +1265,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0009</t>
     </r>
@@ -1158,9 +1287,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0050</t>
     </r>
@@ -1168,9 +1299,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0012</t>
     </r>
@@ -1185,9 +1318,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0011</t>
     </r>
@@ -1205,9 +1340,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0038</t>
     </r>
@@ -1222,9 +1359,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0007</t>
     </r>
@@ -1239,9 +1378,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0030</t>
     </r>
@@ -1256,9 +1397,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0032</t>
     </r>
@@ -1276,9 +1419,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0003</t>
     </r>
@@ -1286,9 +1431,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0002</t>
     </r>
@@ -1306,9 +1453,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0011</t>
     </r>
@@ -1323,9 +1472,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0008</t>
     </r>
@@ -1340,9 +1491,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0039</t>
     </r>
@@ -1350,9 +1503,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0040</t>
     </r>
@@ -1370,9 +1525,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0024</t>
     </r>
@@ -1387,9 +1544,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0033</t>
     </r>
@@ -1407,9 +1566,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0007</t>
     </r>
@@ -1424,9 +1585,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0016</t>
     </r>
@@ -1444,9 +1607,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0006</t>
     </r>
@@ -1464,9 +1629,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0017</t>
     </r>
@@ -1474,9 +1641,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0004</t>
     </r>
@@ -1494,9 +1663,11 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Arial, Verdana, Helvetica, sans-serif"/>
-        <color rgb="FF1155CC"/>
-        <u/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
       </rPr>
       <t>R69-0014</t>
     </r>
@@ -1505,26 +1676,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF333333"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF1155CC"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1532,7 +1711,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1554,69 +1733,70 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="14" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1806,21 +1986,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G82"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="20.63"/>
-    <col customWidth="1" min="2" max="2" width="36.25"/>
+    <col min="1" max="1" width="44.7109375" customWidth="1"/>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1843,7 +2026,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1851,7 +2034,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="4">
-        <v>2270.0</v>
+        <v>2270</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>9</v>
@@ -1860,13 +2043,13 @@
         <v>10</v>
       </c>
       <c r="F2" s="6">
-        <v>46087.0</v>
+        <v>46087</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -1874,7 +2057,7 @@
         <v>13</v>
       </c>
       <c r="C3" s="9">
-        <v>77230.0</v>
+        <v>77230</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>14</v>
@@ -1883,13 +2066,13 @@
         <v>15</v>
       </c>
       <c r="F3" s="10">
-        <v>46084.0</v>
+        <v>46084</v>
       </c>
       <c r="G3" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
@@ -1897,7 +2080,7 @@
         <v>17</v>
       </c>
       <c r="C4" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>18</v>
@@ -1906,13 +2089,13 @@
         <v>19</v>
       </c>
       <c r="F4" s="6">
-        <v>46079.0</v>
+        <v>46079</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>20</v>
       </c>
@@ -1920,7 +2103,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="9">
-        <v>92110.0</v>
+        <v>92110</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>22</v>
@@ -1929,13 +2112,13 @@
         <v>23</v>
       </c>
       <c r="F5" s="10">
-        <v>46069.0</v>
+        <v>46069</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>24</v>
       </c>
@@ -1943,7 +2126,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>18</v>
@@ -1952,13 +2135,13 @@
         <v>26</v>
       </c>
       <c r="F6" s="6">
-        <v>46062.0</v>
+        <v>46062</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>27</v>
       </c>
@@ -1966,7 +2149,7 @@
         <v>28</v>
       </c>
       <c r="C7" s="9">
-        <v>2270.0</v>
+        <v>2270</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>29</v>
@@ -1975,13 +2158,13 @@
         <v>30</v>
       </c>
       <c r="F7" s="10">
-        <v>46000.0</v>
+        <v>46000</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>31</v>
       </c>
@@ -1989,7 +2172,7 @@
         <v>32</v>
       </c>
       <c r="C8" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>18</v>
@@ -1998,13 +2181,13 @@
         <v>33</v>
       </c>
       <c r="F8" s="11">
-        <v>45982.0</v>
+        <v>45982</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>34</v>
       </c>
@@ -2012,7 +2195,7 @@
         <v>35</v>
       </c>
       <c r="C9" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>36</v>
@@ -2021,13 +2204,13 @@
         <v>37</v>
       </c>
       <c r="F9" s="12">
-        <v>45980.0</v>
+        <v>45980</v>
       </c>
       <c r="G9" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
@@ -2035,7 +2218,7 @@
         <v>39</v>
       </c>
       <c r="C10" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>40</v>
@@ -2044,13 +2227,13 @@
         <v>41</v>
       </c>
       <c r="F10" s="11">
-        <v>45971.0</v>
+        <v>45971</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>42</v>
       </c>
@@ -2058,7 +2241,7 @@
         <v>43</v>
       </c>
       <c r="C11" s="9">
-        <v>2870.0</v>
+        <v>2870</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>44</v>
@@ -2067,13 +2250,13 @@
         <v>45</v>
       </c>
       <c r="F11" s="10">
-        <v>45968.0</v>
+        <v>45968</v>
       </c>
       <c r="G11" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>46</v>
       </c>
@@ -2081,7 +2264,7 @@
         <v>47</v>
       </c>
       <c r="C12" s="4">
-        <v>2250.0</v>
+        <v>2250</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>48</v>
@@ -2090,13 +2273,13 @@
         <v>49</v>
       </c>
       <c r="F12" s="11">
-        <v>45954.0</v>
+        <v>45954</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>50</v>
       </c>
@@ -2104,7 +2287,7 @@
         <v>51</v>
       </c>
       <c r="C13" s="9">
-        <v>67500.0</v>
+        <v>67500</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>52</v>
@@ -2113,13 +2296,13 @@
         <v>53</v>
       </c>
       <c r="F13" s="12">
-        <v>45953.0</v>
+        <v>45953</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>54</v>
       </c>
@@ -2127,7 +2310,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="4">
-        <v>2410.0</v>
+        <v>2410</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>56</v>
@@ -2136,13 +2319,13 @@
         <v>57</v>
       </c>
       <c r="F14" s="11">
-        <v>45940.0</v>
+        <v>45940</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>58</v>
       </c>
@@ -2150,7 +2333,7 @@
         <v>59</v>
       </c>
       <c r="C15" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>18</v>
@@ -2159,13 +2342,13 @@
         <v>60</v>
       </c>
       <c r="F15" s="12">
-        <v>45940.0</v>
+        <v>45940</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>61</v>
       </c>
@@ -2173,7 +2356,7 @@
         <v>62</v>
       </c>
       <c r="C16" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>18</v>
@@ -2182,13 +2365,13 @@
         <v>63</v>
       </c>
       <c r="F16" s="6">
-        <v>45932.0</v>
+        <v>45932</v>
       </c>
       <c r="G16" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>64</v>
       </c>
@@ -2196,7 +2379,7 @@
         <v>65</v>
       </c>
       <c r="C17" s="9">
-        <v>2840.0</v>
+        <v>2840</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>66</v>
@@ -2205,13 +2388,13 @@
         <v>67</v>
       </c>
       <c r="F17" s="10">
-        <v>45932.0</v>
+        <v>45932</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>68</v>
       </c>
@@ -2219,7 +2402,7 @@
         <v>69</v>
       </c>
       <c r="C18" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>18</v>
@@ -2228,13 +2411,13 @@
         <v>70</v>
       </c>
       <c r="F18" s="6">
-        <v>45894.0</v>
+        <v>45894</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>71</v>
       </c>
@@ -2242,7 +2425,7 @@
         <v>72</v>
       </c>
       <c r="C19" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>18</v>
@@ -2251,13 +2434,13 @@
         <v>73</v>
       </c>
       <c r="F19" s="10">
-        <v>45894.0</v>
+        <v>45894</v>
       </c>
       <c r="G19" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>74</v>
       </c>
@@ -2265,7 +2448,7 @@
         <v>75</v>
       </c>
       <c r="C20" s="4">
-        <v>2160.0</v>
+        <v>2160</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>76</v>
@@ -2274,13 +2457,13 @@
         <v>77</v>
       </c>
       <c r="F20" s="6">
-        <v>45888.0</v>
+        <v>45888</v>
       </c>
       <c r="G20" s="6">
-        <v>45888.0</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>45888</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>78</v>
       </c>
@@ -2288,7 +2471,7 @@
         <v>79</v>
       </c>
       <c r="C21" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>18</v>
@@ -2297,13 +2480,13 @@
         <v>80</v>
       </c>
       <c r="F21" s="10">
-        <v>45881.0</v>
+        <v>45881</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>81</v>
       </c>
@@ -2311,7 +2494,7 @@
         <v>82</v>
       </c>
       <c r="C22" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>18</v>
@@ -2320,13 +2503,13 @@
         <v>83</v>
       </c>
       <c r="F22" s="6">
-        <v>45870.0</v>
+        <v>45870</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>84</v>
       </c>
@@ -2334,7 +2517,7 @@
         <v>85</v>
       </c>
       <c r="C23" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>18</v>
@@ -2343,13 +2526,13 @@
         <v>86</v>
       </c>
       <c r="F23" s="10">
-        <v>45870.0</v>
+        <v>45870</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>87</v>
       </c>
@@ -2357,7 +2540,7 @@
         <v>88</v>
       </c>
       <c r="C24" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>18</v>
@@ -2366,13 +2549,13 @@
         <v>89</v>
       </c>
       <c r="F24" s="6">
-        <v>45863.0</v>
+        <v>45863</v>
       </c>
       <c r="G24" s="6">
-        <v>46087.0</v>
-      </c>
-    </row>
-    <row r="25">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>90</v>
       </c>
@@ -2380,7 +2563,7 @@
         <v>91</v>
       </c>
       <c r="C25" s="9">
-        <v>77120.0</v>
+        <v>77120</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>92</v>
@@ -2389,13 +2572,13 @@
         <v>93</v>
       </c>
       <c r="F25" s="10">
-        <v>45845.0</v>
+        <v>45845</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>94</v>
       </c>
@@ -2403,7 +2586,7 @@
         <v>95</v>
       </c>
       <c r="C26" s="4">
-        <v>49070.0</v>
+        <v>49070</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>96</v>
@@ -2412,13 +2595,13 @@
         <v>97</v>
       </c>
       <c r="F26" s="6">
-        <v>45839.0</v>
+        <v>45839</v>
       </c>
       <c r="G26" s="11">
-        <v>45951.0</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>45951</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>98</v>
       </c>
@@ -2426,7 +2609,7 @@
         <v>99</v>
       </c>
       <c r="C27" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>18</v>
@@ -2435,13 +2618,13 @@
         <v>100</v>
       </c>
       <c r="F27" s="10">
-        <v>45804.0</v>
+        <v>45804</v>
       </c>
       <c r="G27" s="10">
-        <v>45903.0</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>45903</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>101</v>
       </c>
@@ -2449,7 +2632,7 @@
         <v>102</v>
       </c>
       <c r="C28" s="4">
-        <v>2340.0</v>
+        <v>2340</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>103</v>
@@ -2458,13 +2641,13 @@
         <v>104</v>
       </c>
       <c r="F28" s="6">
-        <v>45792.0</v>
+        <v>45792</v>
       </c>
       <c r="G28" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>105</v>
       </c>
@@ -2472,7 +2655,7 @@
         <v>106</v>
       </c>
       <c r="C29" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>18</v>
@@ -2481,13 +2664,13 @@
         <v>107</v>
       </c>
       <c r="F29" s="10">
-        <v>45789.0</v>
+        <v>45789</v>
       </c>
       <c r="G29" s="10">
-        <v>45929.0</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>45929</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>108</v>
       </c>
@@ -2495,7 +2678,7 @@
         <v>109</v>
       </c>
       <c r="C30" s="4">
-        <v>2840.0</v>
+        <v>2840</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>110</v>
@@ -2504,13 +2687,13 @@
         <v>111</v>
       </c>
       <c r="F30" s="6">
-        <v>45784.0</v>
+        <v>45784</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>112</v>
       </c>
@@ -2518,7 +2701,7 @@
         <v>113</v>
       </c>
       <c r="C31" s="9">
-        <v>10310.0</v>
+        <v>10310</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>114</v>
@@ -2527,13 +2710,13 @@
         <v>115</v>
       </c>
       <c r="F31" s="10">
-        <v>45772.0</v>
+        <v>45772</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>116</v>
       </c>
@@ -2541,7 +2724,7 @@
         <v>117</v>
       </c>
       <c r="C32" s="4">
-        <v>38280.0</v>
+        <v>38280</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>118</v>
@@ -2550,13 +2733,13 @@
         <v>119</v>
       </c>
       <c r="F32" s="6">
-        <v>45736.0</v>
+        <v>45736</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
         <v>120</v>
       </c>
@@ -2564,7 +2747,7 @@
         <v>121</v>
       </c>
       <c r="C33" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>18</v>
@@ -2573,13 +2756,13 @@
         <v>122</v>
       </c>
       <c r="F33" s="10">
-        <v>45733.0</v>
+        <v>45733</v>
       </c>
       <c r="G33" s="12">
-        <v>45986.0</v>
-      </c>
-    </row>
-    <row r="34">
+        <v>45986</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>123</v>
       </c>
@@ -2587,7 +2770,7 @@
         <v>124</v>
       </c>
       <c r="C34" s="4">
-        <v>2860.0</v>
+        <v>2860</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>125</v>
@@ -2596,13 +2779,13 @@
         <v>126</v>
       </c>
       <c r="F34" s="6">
-        <v>45727.0</v>
+        <v>45727</v>
       </c>
       <c r="G34" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
         <v>127</v>
       </c>
@@ -2610,7 +2793,7 @@
         <v>128</v>
       </c>
       <c r="C35" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D35" s="9" t="s">
         <v>18</v>
@@ -2619,13 +2802,13 @@
         <v>129</v>
       </c>
       <c r="F35" s="10">
-        <v>45722.0</v>
+        <v>45722</v>
       </c>
       <c r="G35" s="10">
-        <v>45814.0</v>
-      </c>
-    </row>
-    <row r="36">
+        <v>45814</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>130</v>
       </c>
@@ -2633,7 +2816,7 @@
         <v>131</v>
       </c>
       <c r="C36" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>18</v>
@@ -2642,13 +2825,13 @@
         <v>132</v>
       </c>
       <c r="F36" s="11">
-        <v>45656.0</v>
+        <v>45656</v>
       </c>
       <c r="G36" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
         <v>133</v>
       </c>
@@ -2656,7 +2839,7 @@
         <v>134</v>
       </c>
       <c r="C37" s="9">
-        <v>14800.0</v>
+        <v>14800</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>135</v>
@@ -2665,13 +2848,13 @@
         <v>136</v>
       </c>
       <c r="F37" s="10">
-        <v>45635.0</v>
+        <v>45635</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>137</v>
       </c>
@@ -2679,7 +2862,7 @@
         <v>138</v>
       </c>
       <c r="C38" s="4">
-        <v>2270.0</v>
+        <v>2270</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>139</v>
@@ -2688,13 +2871,13 @@
         <v>140</v>
       </c>
       <c r="F38" s="6">
-        <v>45630.0</v>
+        <v>45630</v>
       </c>
       <c r="G38" s="6">
-        <v>45891.0</v>
-      </c>
-    </row>
-    <row r="39">
+        <v>45891</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
         <v>141</v>
       </c>
@@ -2702,7 +2885,7 @@
         <v>142</v>
       </c>
       <c r="C39" s="9">
-        <v>2820.0</v>
+        <v>2820</v>
       </c>
       <c r="D39" s="9" t="s">
         <v>143</v>
@@ -2711,13 +2894,13 @@
         <v>144</v>
       </c>
       <c r="F39" s="12">
-        <v>45625.0</v>
+        <v>45625</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>145</v>
       </c>
@@ -2725,7 +2908,7 @@
         <v>146</v>
       </c>
       <c r="C40" s="4">
-        <v>2860.0</v>
+        <v>2860</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>147</v>
@@ -2734,13 +2917,13 @@
         <v>148</v>
       </c>
       <c r="F40" s="11">
-        <v>45625.0</v>
+        <v>45625</v>
       </c>
       <c r="G40" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
         <v>149</v>
       </c>
@@ -2748,7 +2931,7 @@
         <v>150</v>
       </c>
       <c r="C41" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>18</v>
@@ -2757,13 +2940,13 @@
         <v>151</v>
       </c>
       <c r="F41" s="12">
-        <v>45621.0</v>
+        <v>45621</v>
       </c>
       <c r="G41" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>152</v>
       </c>
@@ -2771,7 +2954,7 @@
         <v>153</v>
       </c>
       <c r="C42" s="4">
-        <v>2100.0</v>
+        <v>2100</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>154</v>
@@ -2780,13 +2963,13 @@
         <v>155</v>
       </c>
       <c r="F42" s="11">
-        <v>45616.0</v>
+        <v>45616</v>
       </c>
       <c r="G42" s="6">
-        <v>45735.0</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>45735</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
         <v>156</v>
       </c>
@@ -2794,7 +2977,7 @@
         <v>157</v>
       </c>
       <c r="C43" s="9">
-        <v>2250.0</v>
+        <v>2250</v>
       </c>
       <c r="D43" s="9" t="s">
         <v>158</v>
@@ -2803,13 +2986,13 @@
         <v>159</v>
       </c>
       <c r="F43" s="12">
-        <v>45594.0</v>
+        <v>45594</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>160</v>
       </c>
@@ -2817,7 +3000,7 @@
         <v>161</v>
       </c>
       <c r="C44" s="4">
-        <v>77700.0</v>
+        <v>77700</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>162</v>
@@ -2826,13 +3009,13 @@
         <v>163</v>
       </c>
       <c r="F44" s="11">
-        <v>45587.0</v>
+        <v>45587</v>
       </c>
       <c r="G44" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
         <v>164</v>
       </c>
@@ -2840,7 +3023,7 @@
         <v>165</v>
       </c>
       <c r="C45" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D45" s="9" t="s">
         <v>18</v>
@@ -2849,13 +3032,13 @@
         <v>166</v>
       </c>
       <c r="F45" s="10">
-        <v>45561.0</v>
+        <v>45561</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>167</v>
       </c>
@@ -2863,7 +3046,7 @@
         <v>79</v>
       </c>
       <c r="C46" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D46" s="4" t="s">
         <v>18</v>
@@ -2872,13 +3055,13 @@
         <v>168</v>
       </c>
       <c r="F46" s="6">
-        <v>45536.0</v>
+        <v>45536</v>
       </c>
       <c r="G46" s="6">
-        <v>45880.0</v>
-      </c>
-    </row>
-    <row r="47">
+        <v>45880</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
         <v>169</v>
       </c>
@@ -2886,7 +3069,7 @@
         <v>170</v>
       </c>
       <c r="C47" s="9">
-        <v>2320.0</v>
+        <v>2320</v>
       </c>
       <c r="D47" s="9" t="s">
         <v>171</v>
@@ -2895,13 +3078,13 @@
         <v>172</v>
       </c>
       <c r="F47" s="10">
-        <v>45534.0</v>
+        <v>45534</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>173</v>
       </c>
@@ -2909,7 +3092,7 @@
         <v>174</v>
       </c>
       <c r="C48" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>175</v>
@@ -2918,13 +3101,13 @@
         <v>176</v>
       </c>
       <c r="F48" s="6">
-        <v>45532.0</v>
+        <v>45532</v>
       </c>
       <c r="G48" s="6">
-        <v>45762.0</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>45762</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>177</v>
       </c>
@@ -2932,7 +3115,7 @@
         <v>178</v>
       </c>
       <c r="C49" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D49" s="9" t="s">
         <v>18</v>
@@ -2941,13 +3124,13 @@
         <v>179</v>
       </c>
       <c r="F49" s="10">
-        <v>45532.0</v>
+        <v>45532</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>180</v>
       </c>
@@ -2955,7 +3138,7 @@
         <v>181</v>
       </c>
       <c r="C50" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>18</v>
@@ -2964,13 +3147,13 @@
         <v>182</v>
       </c>
       <c r="F50" s="6">
-        <v>45526.0</v>
+        <v>45526</v>
       </c>
       <c r="G50" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>183</v>
       </c>
@@ -2978,7 +3161,7 @@
         <v>184</v>
       </c>
       <c r="C51" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D51" s="9" t="s">
         <v>18</v>
@@ -2987,13 +3170,13 @@
         <v>185</v>
       </c>
       <c r="F51" s="10">
-        <v>45524.0</v>
+        <v>45524</v>
       </c>
       <c r="G51" s="12">
-        <v>46005.0</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>46005</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>186</v>
       </c>
@@ -3001,7 +3184,7 @@
         <v>187</v>
       </c>
       <c r="C52" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>18</v>
@@ -3010,13 +3193,13 @@
         <v>188</v>
       </c>
       <c r="F52" s="6">
-        <v>45516.0</v>
+        <v>45516</v>
       </c>
       <c r="G52" s="6">
-        <v>45631.0</v>
-      </c>
-    </row>
-    <row r="53">
+        <v>45631</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
         <v>186</v>
       </c>
@@ -3024,7 +3207,7 @@
         <v>187</v>
       </c>
       <c r="C53" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D53" s="9" t="s">
         <v>18</v>
@@ -3033,13 +3216,13 @@
         <v>189</v>
       </c>
       <c r="F53" s="10">
-        <v>45516.0</v>
+        <v>45516</v>
       </c>
       <c r="G53" s="10">
-        <v>45631.0</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>45631</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>190</v>
       </c>
@@ -3047,7 +3230,7 @@
         <v>191</v>
       </c>
       <c r="C54" s="4">
-        <v>66120.0</v>
+        <v>66120</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>192</v>
@@ -3056,13 +3239,13 @@
         <v>193</v>
       </c>
       <c r="F54" s="6">
-        <v>45496.0</v>
+        <v>45496</v>
       </c>
       <c r="G54" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>194</v>
       </c>
@@ -3070,7 +3253,7 @@
         <v>195</v>
       </c>
       <c r="C55" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D55" s="9" t="s">
         <v>18</v>
@@ -3079,13 +3262,13 @@
         <v>196</v>
       </c>
       <c r="F55" s="10">
-        <v>45490.0</v>
+        <v>45490</v>
       </c>
       <c r="G55" s="10">
-        <v>45556.0</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>45556</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>197</v>
       </c>
@@ -3093,7 +3276,7 @@
         <v>198</v>
       </c>
       <c r="C56" s="4">
-        <v>2320.0</v>
+        <v>2320</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>171</v>
@@ -3102,13 +3285,13 @@
         <v>199</v>
       </c>
       <c r="F56" s="6">
-        <v>45489.0</v>
+        <v>45489</v>
       </c>
       <c r="G56" s="6">
-        <v>45900.0</v>
-      </c>
-    </row>
-    <row r="57">
+        <v>45900</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
         <v>200</v>
       </c>
@@ -3116,7 +3299,7 @@
         <v>201</v>
       </c>
       <c r="C57" s="9">
-        <v>60100.0</v>
+        <v>60100</v>
       </c>
       <c r="D57" s="9" t="s">
         <v>202</v>
@@ -3125,13 +3308,13 @@
         <v>203</v>
       </c>
       <c r="F57" s="10">
-        <v>45474.0</v>
+        <v>45474</v>
       </c>
       <c r="G57" s="10">
-        <v>45535.0</v>
-      </c>
-    </row>
-    <row r="58">
+        <v>45535</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>204</v>
       </c>
@@ -3139,7 +3322,7 @@
         <v>205</v>
       </c>
       <c r="C58" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D58" s="4" t="s">
         <v>18</v>
@@ -3148,13 +3331,13 @@
         <v>206</v>
       </c>
       <c r="F58" s="6">
-        <v>45470.0</v>
+        <v>45470</v>
       </c>
       <c r="G58" s="11">
-        <v>46001.0</v>
-      </c>
-    </row>
-    <row r="59">
+        <v>46001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
         <v>207</v>
       </c>
@@ -3162,7 +3345,7 @@
         <v>208</v>
       </c>
       <c r="C59" s="9">
-        <v>51100.0</v>
+        <v>51100</v>
       </c>
       <c r="D59" s="9" t="s">
         <v>209</v>
@@ -3171,13 +3354,13 @@
         <v>210</v>
       </c>
       <c r="F59" s="10">
-        <v>45470.0</v>
+        <v>45470</v>
       </c>
       <c r="G59" s="10">
-        <v>46053.0</v>
-      </c>
-    </row>
-    <row r="60">
+        <v>46053</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>211</v>
       </c>
@@ -3185,7 +3368,7 @@
         <v>212</v>
       </c>
       <c r="C60" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D60" s="4" t="s">
         <v>18</v>
@@ -3194,13 +3377,13 @@
         <v>213</v>
       </c>
       <c r="F60" s="6">
-        <v>45450.0</v>
+        <v>45450</v>
       </c>
       <c r="G60" s="6">
-        <v>45829.0</v>
-      </c>
-    </row>
-    <row r="61">
+        <v>45829</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
         <v>214</v>
       </c>
@@ -3208,7 +3391,7 @@
         <v>215</v>
       </c>
       <c r="C61" s="9">
-        <v>2840.0</v>
+        <v>2840</v>
       </c>
       <c r="D61" s="9" t="s">
         <v>216</v>
@@ -3217,13 +3400,13 @@
         <v>217</v>
       </c>
       <c r="F61" s="10">
-        <v>45450.0</v>
+        <v>45450</v>
       </c>
       <c r="G61" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>218</v>
       </c>
@@ -3231,7 +3414,7 @@
         <v>219</v>
       </c>
       <c r="C62" s="4">
-        <v>2350.0</v>
+        <v>2350</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>220</v>
@@ -3240,13 +3423,13 @@
         <v>221</v>
       </c>
       <c r="F62" s="6">
-        <v>45436.0</v>
+        <v>45436</v>
       </c>
       <c r="G62" s="6">
-        <v>45521.0</v>
-      </c>
-    </row>
-    <row r="63">
+        <v>45521</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
         <v>58</v>
       </c>
@@ -3254,7 +3437,7 @@
         <v>59</v>
       </c>
       <c r="C63" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D63" s="9" t="s">
         <v>18</v>
@@ -3263,13 +3446,13 @@
         <v>222</v>
       </c>
       <c r="F63" s="10">
-        <v>45429.0</v>
+        <v>45429</v>
       </c>
       <c r="G63" s="10">
-        <v>45939.0</v>
-      </c>
-    </row>
-    <row r="64">
+        <v>45939</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>223</v>
       </c>
@@ -3277,7 +3460,7 @@
         <v>224</v>
       </c>
       <c r="C64" s="4">
-        <v>2270.0</v>
+        <v>2270</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>139</v>
@@ -3286,13 +3469,13 @@
         <v>225</v>
       </c>
       <c r="F64" s="6">
-        <v>45426.0</v>
+        <v>45426</v>
       </c>
       <c r="G64" s="11">
-        <v>45991.0</v>
-      </c>
-    </row>
-    <row r="65">
+        <v>45991</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
         <v>226</v>
       </c>
@@ -3300,7 +3483,7 @@
         <v>227</v>
       </c>
       <c r="C65" s="9">
-        <v>97434.0</v>
+        <v>97434</v>
       </c>
       <c r="D65" s="9" t="s">
         <v>228</v>
@@ -3309,13 +3492,13 @@
         <v>229</v>
       </c>
       <c r="F65" s="10">
-        <v>45413.0</v>
+        <v>45413</v>
       </c>
       <c r="G65" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>230</v>
       </c>
@@ -3323,7 +3506,7 @@
         <v>231</v>
       </c>
       <c r="C66" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D66" s="4" t="s">
         <v>18</v>
@@ -3332,13 +3515,13 @@
         <v>232</v>
       </c>
       <c r="F66" s="6">
-        <v>45413.0</v>
+        <v>45413</v>
       </c>
       <c r="G66" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
         <v>233</v>
       </c>
@@ -3346,7 +3529,7 @@
         <v>234</v>
       </c>
       <c r="C67" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D67" s="9" t="s">
         <v>18</v>
@@ -3355,13 +3538,13 @@
         <v>235</v>
       </c>
       <c r="F67" s="10">
-        <v>45371.0</v>
+        <v>45371</v>
       </c>
       <c r="G67" s="10">
-        <v>46081.0</v>
-      </c>
-    </row>
-    <row r="68">
+        <v>46081</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>236</v>
       </c>
@@ -3369,7 +3552,7 @@
         <v>237</v>
       </c>
       <c r="C68" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>18</v>
@@ -3378,13 +3561,13 @@
         <v>238</v>
       </c>
       <c r="F68" s="6">
-        <v>45370.0</v>
+        <v>45370</v>
       </c>
       <c r="G68" s="6">
-        <v>45467.0</v>
-      </c>
-    </row>
-    <row r="69">
+        <v>45467</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
         <v>239</v>
       </c>
@@ -3392,7 +3575,7 @@
         <v>240</v>
       </c>
       <c r="C69" s="9">
-        <v>2840.0</v>
+        <v>2840</v>
       </c>
       <c r="D69" s="9" t="s">
         <v>241</v>
@@ -3401,13 +3584,13 @@
         <v>242</v>
       </c>
       <c r="F69" s="10">
-        <v>45348.0</v>
+        <v>45348</v>
       </c>
       <c r="G69" s="10">
-        <v>45913.0</v>
-      </c>
-    </row>
-    <row r="70">
+        <v>45913</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>239</v>
       </c>
@@ -3415,7 +3598,7 @@
         <v>240</v>
       </c>
       <c r="C70" s="4">
-        <v>2840.0</v>
+        <v>2840</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>241</v>
@@ -3424,13 +3607,13 @@
         <v>243</v>
       </c>
       <c r="F70" s="6">
-        <v>45348.0</v>
+        <v>45348</v>
       </c>
       <c r="G70" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
         <v>244</v>
       </c>
@@ -3438,7 +3621,7 @@
         <v>245</v>
       </c>
       <c r="C71" s="9">
-        <v>2320.0</v>
+        <v>2320</v>
       </c>
       <c r="D71" s="9" t="s">
         <v>246</v>
@@ -3447,13 +3630,13 @@
         <v>247</v>
       </c>
       <c r="F71" s="10">
-        <v>45345.0</v>
+        <v>45345</v>
       </c>
       <c r="G71" s="10">
-        <v>45412.0</v>
-      </c>
-    </row>
-    <row r="72">
+        <v>45412</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>248</v>
       </c>
@@ -3461,7 +3644,7 @@
         <v>249</v>
       </c>
       <c r="C72" s="4">
-        <v>2860.0</v>
+        <v>2860</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>147</v>
@@ -3470,13 +3653,13 @@
         <v>250</v>
       </c>
       <c r="F72" s="6">
-        <v>45315.0</v>
+        <v>45315</v>
       </c>
       <c r="G72" s="11">
-        <v>45626.0</v>
-      </c>
-    </row>
-    <row r="73">
+        <v>45626</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
         <v>251</v>
       </c>
@@ -3484,7 +3667,7 @@
         <v>252</v>
       </c>
       <c r="C73" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D73" s="9" t="s">
         <v>18</v>
@@ -3493,13 +3676,13 @@
         <v>253</v>
       </c>
       <c r="F73" s="12">
-        <v>45282.0</v>
+        <v>45282</v>
       </c>
       <c r="G73" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>251</v>
       </c>
@@ -3507,7 +3690,7 @@
         <v>252</v>
       </c>
       <c r="C74" s="4">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>18</v>
@@ -3516,13 +3699,13 @@
         <v>254</v>
       </c>
       <c r="F74" s="11">
-        <v>45282.0</v>
+        <v>45282</v>
       </c>
       <c r="G74" s="6">
-        <v>45869.0</v>
-      </c>
-    </row>
-    <row r="75">
+        <v>45869</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
         <v>255</v>
       </c>
@@ -3530,7 +3713,7 @@
         <v>256</v>
       </c>
       <c r="C75" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D75" s="9" t="s">
         <v>257</v>
@@ -3539,13 +3722,13 @@
         <v>258</v>
       </c>
       <c r="F75" s="12">
-        <v>45279.0</v>
+        <v>45279</v>
       </c>
       <c r="G75" s="10">
-        <v>45433.0</v>
-      </c>
-    </row>
-    <row r="76">
+        <v>45433</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>259</v>
       </c>
@@ -3553,7 +3736,7 @@
         <v>260</v>
       </c>
       <c r="C76" s="4">
-        <v>2270.0</v>
+        <v>2270</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>29</v>
@@ -3562,13 +3745,13 @@
         <v>261</v>
       </c>
       <c r="F76" s="11">
-        <v>45253.0</v>
+        <v>45253</v>
       </c>
       <c r="G76" s="11">
-        <v>45991.0</v>
-      </c>
-    </row>
-    <row r="77">
+        <v>45991</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
         <v>262</v>
       </c>
@@ -3576,7 +3759,7 @@
         <v>263</v>
       </c>
       <c r="C77" s="9">
-        <v>59148.0</v>
+        <v>59148</v>
       </c>
       <c r="D77" s="9" t="s">
         <v>264</v>
@@ -3585,13 +3768,13 @@
         <v>265</v>
       </c>
       <c r="F77" s="12">
-        <v>45247.0</v>
+        <v>45247</v>
       </c>
       <c r="G77" s="10">
-        <v>45380.0</v>
-      </c>
-    </row>
-    <row r="78">
+        <v>45380</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>266</v>
       </c>
@@ -3599,7 +3782,7 @@
         <v>267</v>
       </c>
       <c r="C78" s="4">
-        <v>51100.0</v>
+        <v>51100</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>209</v>
@@ -3608,13 +3791,13 @@
         <v>268</v>
       </c>
       <c r="F78" s="6">
-        <v>45239.0</v>
+        <v>45239</v>
       </c>
       <c r="G78" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
         <v>269</v>
       </c>
@@ -3622,7 +3805,7 @@
         <v>270</v>
       </c>
       <c r="C79" s="9">
-        <v>2200.0</v>
+        <v>2200</v>
       </c>
       <c r="D79" s="9" t="s">
         <v>271</v>
@@ -3631,13 +3814,13 @@
         <v>272</v>
       </c>
       <c r="F79" s="12">
-        <v>45222.0</v>
+        <v>45222</v>
       </c>
       <c r="G79" s="10">
-        <v>45361.0</v>
-      </c>
-    </row>
-    <row r="80">
+        <v>45361</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>273</v>
       </c>
@@ -3645,7 +3828,7 @@
         <v>274</v>
       </c>
       <c r="C80" s="4">
-        <v>2870.0</v>
+        <v>2870</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>275</v>
@@ -3654,13 +3837,13 @@
         <v>276</v>
       </c>
       <c r="F80" s="11">
-        <v>45212.0</v>
+        <v>45212</v>
       </c>
       <c r="G80" s="6">
-        <v>45565.0</v>
-      </c>
-    </row>
-    <row r="81">
+        <v>45565</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
         <v>84</v>
       </c>
@@ -3668,7 +3851,7 @@
         <v>85</v>
       </c>
       <c r="C81" s="9">
-        <v>2000.0</v>
+        <v>2000</v>
       </c>
       <c r="D81" s="9" t="s">
         <v>18</v>
@@ -3677,13 +3860,13 @@
         <v>277</v>
       </c>
       <c r="F81" s="10">
-        <v>45208.0</v>
+        <v>45208</v>
       </c>
       <c r="G81" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>278</v>
       </c>
@@ -3691,7 +3874,7 @@
         <v>279</v>
       </c>
       <c r="C82" s="4">
-        <v>2860.0</v>
+        <v>2860</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>280</v>
@@ -3700,96 +3883,96 @@
         <v>281</v>
       </c>
       <c r="F82" s="6">
-        <v>45159.0</v>
+        <v>45159</v>
       </c>
       <c r="G82" s="6">
-        <v>45516.0</v>
+        <v>45516</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="E2"/>
-    <hyperlink r:id="rId2" ref="E3"/>
-    <hyperlink r:id="rId3" ref="E4"/>
-    <hyperlink r:id="rId4" ref="E5"/>
-    <hyperlink r:id="rId5" ref="E6"/>
-    <hyperlink r:id="rId6" ref="E7"/>
-    <hyperlink r:id="rId7" ref="E8"/>
-    <hyperlink r:id="rId8" ref="E9"/>
-    <hyperlink r:id="rId9" ref="E10"/>
-    <hyperlink r:id="rId10" ref="E11"/>
-    <hyperlink r:id="rId11" ref="E12"/>
-    <hyperlink r:id="rId12" ref="E13"/>
-    <hyperlink r:id="rId13" ref="E14"/>
-    <hyperlink r:id="rId14" ref="E15"/>
-    <hyperlink r:id="rId15" ref="E16"/>
-    <hyperlink r:id="rId16" ref="E17"/>
-    <hyperlink r:id="rId17" ref="E18"/>
-    <hyperlink r:id="rId18" ref="E19"/>
-    <hyperlink r:id="rId19" ref="E20"/>
-    <hyperlink r:id="rId20" ref="E21"/>
-    <hyperlink r:id="rId21" ref="E22"/>
-    <hyperlink r:id="rId22" ref="E23"/>
-    <hyperlink r:id="rId23" ref="E24"/>
-    <hyperlink r:id="rId24" ref="E25"/>
-    <hyperlink r:id="rId25" ref="E26"/>
-    <hyperlink r:id="rId26" ref="E27"/>
-    <hyperlink r:id="rId27" ref="E28"/>
-    <hyperlink r:id="rId28" ref="E29"/>
-    <hyperlink r:id="rId29" ref="E30"/>
-    <hyperlink r:id="rId30" ref="E31"/>
-    <hyperlink r:id="rId31" ref="E32"/>
-    <hyperlink r:id="rId32" ref="E33"/>
-    <hyperlink r:id="rId33" ref="E34"/>
-    <hyperlink r:id="rId34" ref="E35"/>
-    <hyperlink r:id="rId35" ref="E36"/>
-    <hyperlink r:id="rId36" ref="E37"/>
-    <hyperlink r:id="rId37" ref="E38"/>
-    <hyperlink r:id="rId38" ref="E39"/>
-    <hyperlink r:id="rId39" ref="E40"/>
-    <hyperlink r:id="rId40" ref="E41"/>
-    <hyperlink r:id="rId41" ref="E42"/>
-    <hyperlink r:id="rId42" ref="E43"/>
-    <hyperlink r:id="rId43" ref="E44"/>
-    <hyperlink r:id="rId44" ref="E45"/>
-    <hyperlink r:id="rId45" ref="E46"/>
-    <hyperlink r:id="rId46" ref="E47"/>
-    <hyperlink r:id="rId47" ref="E48"/>
-    <hyperlink r:id="rId48" ref="E49"/>
-    <hyperlink r:id="rId49" ref="E50"/>
-    <hyperlink r:id="rId50" ref="E51"/>
-    <hyperlink r:id="rId51" ref="E52"/>
-    <hyperlink r:id="rId52" ref="E53"/>
-    <hyperlink r:id="rId53" ref="E54"/>
-    <hyperlink r:id="rId54" ref="E55"/>
-    <hyperlink r:id="rId55" ref="E56"/>
-    <hyperlink r:id="rId56" ref="E57"/>
-    <hyperlink r:id="rId57" ref="E58"/>
-    <hyperlink r:id="rId58" ref="E59"/>
-    <hyperlink r:id="rId59" ref="E60"/>
-    <hyperlink r:id="rId60" ref="E61"/>
-    <hyperlink r:id="rId61" ref="E62"/>
-    <hyperlink r:id="rId62" ref="E63"/>
-    <hyperlink r:id="rId63" ref="E64"/>
-    <hyperlink r:id="rId64" ref="E65"/>
-    <hyperlink r:id="rId65" ref="E66"/>
-    <hyperlink r:id="rId66" ref="E67"/>
-    <hyperlink r:id="rId67" ref="E68"/>
-    <hyperlink r:id="rId68" ref="E69"/>
-    <hyperlink r:id="rId69" ref="E70"/>
-    <hyperlink r:id="rId70" ref="E71"/>
-    <hyperlink r:id="rId71" ref="E72"/>
-    <hyperlink r:id="rId72" ref="E73"/>
-    <hyperlink r:id="rId73" ref="E74"/>
-    <hyperlink r:id="rId74" ref="E75"/>
-    <hyperlink r:id="rId75" ref="E76"/>
-    <hyperlink r:id="rId76" ref="E77"/>
-    <hyperlink r:id="rId77" ref="E78"/>
-    <hyperlink r:id="rId78" ref="E79"/>
-    <hyperlink r:id="rId79" ref="E80"/>
-    <hyperlink r:id="rId80" ref="E81"/>
-    <hyperlink r:id="rId81" ref="E82"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="E7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="E8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="E9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="E10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="E11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="E12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="E15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="E16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="E19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="E22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="E24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="E25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="E26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="E27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="E28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="E29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="E30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="E31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="E32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="E33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="E34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="E35" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="E36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="E37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="E38" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="E39" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="E40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="E41" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="E42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="E43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="E44" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="E45" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="E46" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="E47" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="E48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="E49" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="E50" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="E51" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="E52" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="E53" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="E54" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="E55" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="E56" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="E57" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="E58" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="E59" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="E60" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="E61" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="E62" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="E63" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="E64" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="E65" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="E66" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="E67" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="E68" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="E69" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="E70" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="E71" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="E72" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="E73" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="E74" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="E75" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="E76" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="E77" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="E78" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="E79" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="E80" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="E81" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="E82" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
   </hyperlinks>
-  <drawing r:id="rId82"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>